<commit_message>
Actualizado Formateo Excel en función de la Prioridad
</commit_message>
<xml_diff>
--- a/customer-stories/Customer_Stories_PlanB.xlsx
+++ b/customer-stories/Customer_Stories_PlanB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mattp\dev\school\3-GISI\ISW-Practica\customer-stories\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F76862E-EC88-4E63-86DF-23295D001E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{985E4E03-3AEB-4303-96EC-559D273C4A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="739" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1601" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="292">
   <si>
     <t>#</t>
   </si>
@@ -947,6 +947,18 @@
   </si>
   <si>
     <t>LUC10</t>
+  </si>
+  <si>
+    <t>M</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>IM</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1108,1928 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="192">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2415,6 +4348,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="149" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="148" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="147" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
   </hyperlinks>
@@ -2580,6 +4524,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="146" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="145" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="144" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
   </hyperlinks>
@@ -2745,6 +4700,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="143" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="142" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="141" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
   </hyperlinks>
@@ -2910,6 +4876,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="140" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="139" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="138" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0C00-000000000000}"/>
   </hyperlinks>
@@ -3075,6 +5052,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="137" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="136" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="135" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0D00-000000000000}"/>
   </hyperlinks>
@@ -3240,6 +5228,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="134" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="133" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="132" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0E00-000000000000}"/>
   </hyperlinks>
@@ -3405,6 +5404,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="131" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="130" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="129" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0F00-000000000000}"/>
   </hyperlinks>
@@ -3570,6 +5580,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="128" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="127" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="126" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1000-000000000000}"/>
   </hyperlinks>
@@ -3735,6 +5756,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="125" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="124" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="123" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1100-000000000000}"/>
   </hyperlinks>
@@ -3900,6 +5932,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="122" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="121" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="120" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1200-000000000000}"/>
   </hyperlinks>
@@ -4065,6 +6108,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="173" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="172" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="171" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
   </hyperlinks>
@@ -4230,6 +6284,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="119" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="118" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="117" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1300-000000000000}"/>
   </hyperlinks>
@@ -4395,6 +6460,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="116" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="115" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="114" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1400-000000000000}"/>
   </hyperlinks>
@@ -4560,6 +6636,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="113" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="112" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="111" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1500-000000000000}"/>
   </hyperlinks>
@@ -4727,6 +6814,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="110" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="109" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="108" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1600-000000000000}"/>
   </hyperlinks>
@@ -4890,6 +6988,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="107" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="106" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="105" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1700-000000000000}"/>
   </hyperlinks>
@@ -5057,6 +7166,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="104" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="103" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="102" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1800-000000000000}"/>
   </hyperlinks>
@@ -5224,6 +7344,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="101" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="100" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="99" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1900-000000000000}"/>
   </hyperlinks>
@@ -5387,6 +7518,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="98" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="97" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="96" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1A00-000000000000}"/>
   </hyperlinks>
@@ -5452,21 +7594,27 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>290</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>223</v>
+      </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="8">
+        <v>13</v>
+      </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -5550,6 +7698,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="95" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="94" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="93" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1B00-000000000000}"/>
   </hyperlinks>
@@ -5717,6 +7876,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="92" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="91" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="90" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1C00-000000000000}"/>
   </hyperlinks>
@@ -5882,6 +8052,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="170" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="169" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="168" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
@@ -6045,6 +8226,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="89" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="88" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="87" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1D00-000000000000}"/>
   </hyperlinks>
@@ -6110,21 +8302,27 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>289</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="8">
+        <v>7</v>
+      </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -6208,6 +8406,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="86" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="85" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="84" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1E00-000000000000}"/>
   </hyperlinks>
@@ -6371,6 +8580,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="83" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="82" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="81" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-1F00-000000000000}"/>
   </hyperlinks>
@@ -6534,6 +8754,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="80" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="79" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="78" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2000-000000000000}"/>
   </hyperlinks>
@@ -6599,21 +8830,27 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>289</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="8">
+        <v>4</v>
+      </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -6697,6 +8934,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="77" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="76" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="75" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2100-000000000000}"/>
   </hyperlinks>
@@ -6860,6 +9108,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="74" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="73" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="72" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2200-000000000000}"/>
   </hyperlinks>
@@ -7023,6 +9282,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="71" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="70" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="69" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2300-000000000000}"/>
   </hyperlinks>
@@ -7088,21 +9358,27 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>290</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="8">
+        <v>6</v>
+      </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -7186,6 +9462,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="68" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="67" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="66" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2400-000000000000}"/>
   </hyperlinks>
@@ -7349,6 +9636,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="65" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="64" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="63" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2500-000000000000}"/>
   </hyperlinks>
@@ -7512,6 +9810,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="62" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="61" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="60" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2600-000000000000}"/>
   </hyperlinks>
@@ -7677,6 +9986,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="167" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="166" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="165" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
   </hyperlinks>
@@ -7840,6 +10160,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="59" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="58" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="57" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2700-000000000000}"/>
   </hyperlinks>
@@ -8007,6 +10338,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="56" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="55" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="54" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2800-000000000000}"/>
   </hyperlinks>
@@ -8170,6 +10512,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="53" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="52" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="51" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2900-000000000000}"/>
   </hyperlinks>
@@ -8337,6 +10690,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="50" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="49" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="48" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2A00-000000000000}"/>
   </hyperlinks>
@@ -8500,6 +10864,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="47" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="46" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="45" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2B00-000000000000}"/>
   </hyperlinks>
@@ -8565,7 +10940,9 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>288</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -8663,6 +11040,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="44" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="43" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="42" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2C00-000000000000}"/>
   </hyperlinks>
@@ -8826,6 +11214,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="41" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="40" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="39" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2D00-000000000000}"/>
   </hyperlinks>
@@ -8989,6 +11388,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="38" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="37" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="36" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2E00-000000000000}"/>
   </hyperlinks>
@@ -9152,6 +11562,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="35" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="34" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="33" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-2F00-000000000000}"/>
   </hyperlinks>
@@ -9315,6 +11736,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="32" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="31" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3000-000000000000}"/>
   </hyperlinks>
@@ -9480,6 +11912,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="164" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="163" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="162" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
@@ -9647,6 +12090,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="29" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="28" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="27" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3100-000000000000}"/>
   </hyperlinks>
@@ -9814,6 +12268,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="26" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3200-000000000000}"/>
   </hyperlinks>
@@ -9977,6 +12442,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="23" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="22" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="21" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3300-000000000000}"/>
   </hyperlinks>
@@ -10140,6 +12616,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3400-000000000000}"/>
   </hyperlinks>
@@ -10303,6 +12790,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="17" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3500-000000000000}"/>
   </hyperlinks>
@@ -10470,6 +12968,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="14" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="13" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="12" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3600-000000000000}"/>
   </hyperlinks>
@@ -10633,6 +13142,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3700-000000000000}"/>
   </hyperlinks>
@@ -10800,6 +13320,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3800-000000000000}"/>
   </hyperlinks>
@@ -10865,21 +13396,27 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>289</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="6"/>
+      <c r="B7" s="6" t="s">
+        <v>226</v>
+      </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B8" s="6"/>
+      <c r="B8" s="8">
+        <v>3</v>
+      </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" spans="1:3" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -10963,6 +13500,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3900-000000000000}"/>
   </hyperlinks>
@@ -11126,11 +13674,22 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-3A00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11291,6 +13850,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="161" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="160" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="159" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
   </hyperlinks>
@@ -11358,7 +13928,9 @@
       <c r="A6" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="6"/>
+      <c r="B6" s="6" t="s">
+        <v>291</v>
+      </c>
       <c r="C6" s="10"/>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -11456,6 +14028,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="158" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="157" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="156" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
   </hyperlinks>
@@ -11621,6 +14204,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="155" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="154" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="153" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
   </hyperlinks>
@@ -11786,6 +14380,17 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="C2:C18"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6">
+    <cfRule type="containsText" dxfId="152" priority="1" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="151" priority="2" operator="containsText" text="N">
+      <formula>NOT(ISERROR(SEARCH("N",B6)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="150" priority="3" operator="containsText" text="M">
+      <formula>NOT(ISERROR(SEARCH("M",B6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="A19" location="Índice!A1" display="↑ Volver al índice" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Excel: FLA05 tareas 4 y 5 hechas (30 min cada una)
</commit_message>
<xml_diff>
--- a/customer-stories/Customer_Stories_PlanB.xlsx
+++ b/customer-stories/Customer_Stories_PlanB.xlsx
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1636" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="335">
   <si>
     <t>#</t>
   </si>
@@ -11608,8 +11608,12 @@
       <c r="B15" s="22" t="s">
         <v>297</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="29"/>
+      <c r="C15" s="17" t="s">
+        <v>294</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>326</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="30" customHeight="1">
       <c r="A16" s="21" t="s">
@@ -11618,8 +11622,12 @@
       <c r="B16" s="22" t="s">
         <v>298</v>
       </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="29"/>
+      <c r="C16" s="17" t="s">
+        <v>294</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>326</v>
+      </c>
     </row>
     <row r="17" spans="1:4" ht="30" customHeight="1">
       <c r="A17" s="21" t="s">

</xml_diff>